<commit_message>
feat: re-evaluate enron with full PA metric set (jaccard_pa, macro_f1_pa, micro_f1_pa)
Enron was originally evaluated before 11 new PartialAbstention metrics were
added to the pipeline. Re-ran evaluate.py + summarize_metrics.py on the
existing merged PKLs (no retraining) to populate the missing columns.

enron_PartialAbstention_summary.csv now has 18 PA metrics (was 7), matching
all other datasets. Also adds scripts/ablations/reeval_enron.sbatch for
reproducibility.
</commit_message>
<xml_diff>
--- a/results/full_enron_split_summary/enron_BinaryVector_summary.xlsx
+++ b/results/full_enron_split_summary/enron_BinaryVector_summary.xlsx
@@ -3880,182 +3880,182 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.7665±0.0322</t>
+          <t>0.7297±0.0357</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.7341±0.0329</t>
+          <t>0.6516±0.0331</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.6992±0.0294</t>
+          <t>0.5787±0.0351</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.6432±0.0294</t>
+          <t>0.4435±0.0273</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.6903±0.0169</t>
+          <t>0.6722±0.0059</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0.5972±0.0186</t>
+          <t>0.4876±0.0112</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0.5353±0.0169</t>
+          <t>0.3098±0.0073</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>0.4265±0.0190</t>
+          <t>0.1755±0.0061</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>0.5227±0.0132</t>
+          <t>0.5832±0.0122</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>0.5173±0.0153</t>
+          <t>0.6076±0.0135</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0.5095±0.0169</t>
+          <t>0.6020±0.0174</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>0.4931±0.0202</t>
+          <t>0.5966±0.0164</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0.5634±0.0108</t>
+          <t>0.5984±0.0056</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>0.5023±0.0147</t>
+          <t>0.4988±0.0079</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>0.4550±0.0131</t>
+          <t>0.3670±0.0077</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>0.3805±0.0136</t>
+          <t>0.2489±0.0062</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>0.9532±0.0015</t>
+          <t>0.9533±0.0012</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>0.9333±0.0025</t>
+          <t>0.9214±0.0016</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>0.9062±0.0043</t>
+          <t>0.8646±0.0035</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>0.8652±0.0067</t>
+          <t>0.7680±0.0054</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>0.4518±0.0106</t>
+          <t>0.4890±0.0071</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>0.3864±0.0141</t>
+          <t>0.3722±0.0087</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>0.3435±0.0126</t>
+          <t>0.2473±0.0069</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>0.2735±0.0118</t>
+          <t>0.1520±0.0046</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>0.1746±0.0260</t>
+          <t>0.2055±0.0264</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>0.1501±0.0119</t>
+          <t>0.1781±0.0074</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>0.1322±0.0079</t>
+          <t>0.1485±0.0056</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>0.1189±0.0084</t>
+          <t>0.1259±0.0035</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>0.2711±0.0342</t>
+          <t>0.2911±0.0341</t>
         </is>
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>0.1617±0.0110</t>
+          <t>0.1602±0.0050</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>0.1250±0.0069</t>
+          <t>0.1217±0.0035</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>0.1026±0.0064</t>
+          <t>0.0967±0.0020</t>
         </is>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>0.1502±0.0236</t>
+          <t>0.1832±0.0243</t>
         </is>
       </c>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>0.1668±0.0227</t>
+          <t>0.2327±0.0243</t>
         </is>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>0.1780±0.0228</t>
+          <t>0.2571±0.0283</t>
         </is>
       </c>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>0.1997±0.0273</t>
+          <t>0.3162±0.0323</t>
         </is>
       </c>
       <c r="AL13" t="inlineStr">
@@ -4065,97 +4065,97 @@
       </c>
       <c r="AM13" t="inlineStr">
         <is>
-          <t>0.9917±0.0026</t>
+          <t>0.9848±0.0048</t>
         </is>
       </c>
       <c r="AN13" t="inlineStr">
         <is>
-          <t>0.9728±0.0054</t>
+          <t>0.9425±0.0089</t>
         </is>
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>0.9379±0.0095</t>
+          <t>0.8500±0.0159</t>
         </is>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>0.5740±0.0096</t>
+          <t>0.6000±0.0063</t>
         </is>
       </c>
       <c r="AQ13" t="inlineStr">
         <is>
-          <t>0.4854±0.0116</t>
+          <t>0.4834±0.0063</t>
         </is>
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>0.3983±0.0119</t>
+          <t>0.3500±0.0074</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>0.3100±0.0132</t>
+          <t>0.2384±0.0053</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>0.6831±0.0148</t>
+          <t>0.6613±0.0109</t>
         </is>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>0.4782±0.0161</t>
+          <t>0.4159±0.0081</t>
         </is>
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>0.3374±0.0146</t>
+          <t>0.2522±0.0058</t>
         </is>
       </c>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>0.2303±0.0123</t>
+          <t>0.1508±0.0038</t>
         </is>
       </c>
       <c r="AX13" t="inlineStr">
         <is>
-          <t>0.4951±0.0101</t>
+          <t>0.5491±0.0050</t>
         </is>
       </c>
       <c r="AY13" t="inlineStr">
         <is>
-          <t>0.4929±0.0092</t>
+          <t>0.5772±0.0089</t>
         </is>
       </c>
       <c r="AZ13" t="inlineStr">
         <is>
-          <t>0.4867±0.0144</t>
+          <t>0.5720±0.0154</t>
         </is>
       </c>
       <c r="BA13" t="inlineStr">
         <is>
-          <t>0.4747±0.0182</t>
+          <t>0.5697±0.0125</t>
         </is>
       </c>
       <c r="BB13" t="inlineStr">
         <is>
-          <t>0.1299±0.0188</t>
+          <t>0.1651±0.0175</t>
         </is>
       </c>
       <c r="BC13" t="inlineStr">
         <is>
-          <t>0.0830±0.0138</t>
+          <t>0.0491±0.0119</t>
         </is>
       </c>
       <c r="BD13" t="inlineStr">
         <is>
-          <t>0.0662±0.0145</t>
+          <t>0.0051±0.0034</t>
         </is>
       </c>
       <c r="BE13" t="inlineStr">
         <is>
-          <t>0.0306±0.0086</t>
+          <t>0.0002±0.0008</t>
         </is>
       </c>
     </row>
@@ -4172,17 +4172,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.8095±0.0261</t>
+          <t>0.8131±0.0296</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.7609±0.0331</t>
+          <t>0.7601±0.0300</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0.6426±0.0296</t>
+          <t>0.6343±0.0304</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -4192,17 +4192,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0.4808±0.0383</t>
+          <t>0.4759±0.0299</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0.3267±0.0318</t>
+          <t>0.3393±0.0210</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>0.1735±0.0153</t>
+          <t>0.1714±0.0147</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -4212,17 +4212,17 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>0.3846±0.0310</t>
+          <t>0.3819±0.0251</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0.3827±0.0362</t>
+          <t>0.3928±0.0244</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>0.4062±0.0417</t>
+          <t>0.4068±0.0342</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -4232,17 +4232,17 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>0.3968±0.0298</t>
+          <t>0.3953±0.0250</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>0.3237±0.0275</t>
+          <t>0.3347±0.0181</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>0.2288±0.0213</t>
+          <t>0.2265±0.0174</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -4252,17 +4252,17 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>0.9391±0.0015</t>
+          <t>0.9394±0.0016</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>0.9130±0.0046</t>
+          <t>0.9152±0.0042</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>0.8431±0.0054</t>
+          <t>0.8408±0.0077</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -4272,17 +4272,17 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>0.2969±0.0244</t>
+          <t>0.2975±0.0219</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>0.2228±0.0204</t>
+          <t>0.2308±0.0146</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>0.1401±0.0142</t>
+          <t>0.1387±0.0119</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -4292,17 +4292,17 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>0.1049±0.0138</t>
+          <t>0.1023±0.0086</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>0.1046±0.0102</t>
+          <t>0.1055±0.0074</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>0.0996±0.0061</t>
+          <t>0.1011±0.0068</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
@@ -4312,17 +4312,17 @@
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>0.1481±0.0257</t>
+          <t>0.1446±0.0185</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>0.1169±0.0150</t>
+          <t>0.1168±0.0108</t>
         </is>
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>0.0871±0.0045</t>
+          <t>0.0880±0.0061</t>
         </is>
       </c>
       <c r="AH14" t="inlineStr">
@@ -4332,17 +4332,17 @@
       </c>
       <c r="AI14" t="inlineStr">
         <is>
-          <t>0.0971±0.0152</t>
+          <t>0.0926±0.0079</t>
         </is>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>0.1216±0.0221</t>
+          <t>0.1232±0.0153</t>
         </is>
       </c>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>0.1794±0.0205</t>
+          <t>0.1843±0.0292</t>
         </is>
       </c>
       <c r="AL14" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>0.9803±0.0088</t>
+          <t>0.9822±0.0114</t>
         </is>
       </c>
       <c r="AP14" t="inlineStr">
@@ -4372,17 +4372,17 @@
       </c>
       <c r="AQ14" t="inlineStr">
         <is>
-          <t>0.4379±0.0224</t>
+          <t>0.4378±0.0200</t>
         </is>
       </c>
       <c r="AR14" t="inlineStr">
         <is>
-          <t>0.3513±0.0240</t>
+          <t>0.3656±0.0192</t>
         </is>
       </c>
       <c r="AS14" t="inlineStr">
         <is>
-          <t>0.2450±0.0187</t>
+          <t>0.2428±0.0158</t>
         </is>
       </c>
       <c r="AT14" t="inlineStr">
@@ -4392,17 +4392,17 @@
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>0.5318±0.0204</t>
+          <t>0.5354±0.0229</t>
         </is>
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>0.3357±0.0252</t>
+          <t>0.3505±0.0234</t>
         </is>
       </c>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>0.1767±0.0128</t>
+          <t>0.1744±0.0126</t>
         </is>
       </c>
       <c r="AX14" t="inlineStr">
@@ -4412,17 +4412,17 @@
       </c>
       <c r="AY14" t="inlineStr">
         <is>
-          <t>0.3731±0.0286</t>
+          <t>0.3706±0.0215</t>
         </is>
       </c>
       <c r="AZ14" t="inlineStr">
         <is>
-          <t>0.3700±0.0326</t>
+          <t>0.3831±0.0230</t>
         </is>
       </c>
       <c r="BA14" t="inlineStr">
         <is>
-          <t>0.3998±0.0370</t>
+          <t>0.3999±0.0259</t>
         </is>
       </c>
       <c r="BB14" t="inlineStr">
@@ -4432,17 +4432,17 @@
       </c>
       <c r="BC14" t="inlineStr">
         <is>
-          <t>0.0476±0.0171</t>
+          <t>0.0523±0.0171</t>
         </is>
       </c>
       <c r="BD14" t="inlineStr">
         <is>
-          <t>0.0120±0.0072</t>
+          <t>0.0093±0.0082</t>
         </is>
       </c>
       <c r="BE14" t="inlineStr">
         <is>
-          <t>0.0000±0.0000</t>
+          <t>0.0004±0.0010</t>
         </is>
       </c>
     </row>

</xml_diff>